<commit_message>
test: update EQL-2 registration result
</commit_message>
<xml_diff>
--- a/casos-de-teste/casos-de-teste-ecommerce.xlsx
+++ b/casos-de-teste/casos-de-teste-ecommerce.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qa-ecommerce-testing\casos-de-teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C9D8C97-0DC0-4DA6-8476-218E8DA252C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99DA248A-D12A-4805-85D8-55468F0916F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{97BBE64D-9E90-40F0-B82D-63AF4B321200}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>ID</t>
   </si>
@@ -88,6 +88,33 @@
   </si>
   <si>
     <t>Página inicial carregou corretamente. Logo, menu de navegação e produtos estavam visíveis. Nenhuma mensagem de erro foi apresentada.</t>
+  </si>
+  <si>
+    <t>Cadastro de novo usuário</t>
+  </si>
+  <si>
+    <t>Usuário não cadastrado no sistema</t>
+  </si>
+  <si>
+    <t>1. Acessar o Automation Exercise.
+2. Acessar a opção de cadastro /login.
+3. Informar nome e e-mail.
+4. Prosseguir com o cadastro.
+5. Preencher os dados obrigatórios.
+6 . Confirmar o cadastro.</t>
+  </si>
+  <si>
+    <t>EQL-2</t>
+  </si>
+  <si>
+    <t>Usuário deve ser cadastrado com sucesso e o sistema deve confirmar a criação da conta</t>
+  </si>
+  <si>
+    <t>Usuário cadastrado com sucesso. Após a confirmação do cadastro, o sistema exibiu a mensagem “Account Created!”, confirmando a criação da conta.</t>
+  </si>
+  <si>
+    <t>EQL-2-cadastro-dados.png
+EQL-2-cadastro-sucesso.png</t>
   </si>
 </sst>
 </file>
@@ -471,11 +498,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93300EE1-EB34-4D2F-ADA0-E6E175CD608D}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.453125" customWidth="1"/>
-    <col min="2" max="2" width="19.90625" customWidth="1"/>
+    <col min="2" max="2" width="22.1796875" customWidth="1"/>
     <col min="3" max="3" width="29.7265625" customWidth="1"/>
     <col min="4" max="4" width="44" style="5" customWidth="1"/>
     <col min="5" max="5" width="29.90625" customWidth="1"/>
@@ -541,7 +568,37 @@
         <v>9</v>
       </c>
     </row>
+    <row r="3" spans="1:9" ht="87" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>